<commit_message>
feat: map URL data content + extract content images from Grasen API
</commit_message>
<xml_diff>
--- a/Grasen_Scraped_Data/Grasen_News_Data.xlsx
+++ b/Grasen_Scraped_Data/Grasen_News_Data.xlsx
@@ -558,7 +558,7 @@
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>https://www.grasen.com/news/ev-charging-management-software</t>
+          <t>https://www.grasen.com/news/ev-charging-management-software-csms</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
@@ -588,7 +588,7 @@
       </c>
       <c r="L2" s="2" t="inlineStr">
         <is>
-          <t>(none — JS-rendered page)</t>
+          <t>(text only — no embedded images)</t>
         </is>
       </c>
     </row>
@@ -650,7 +650,7 @@
       </c>
       <c r="L3" s="3" t="inlineStr">
         <is>
-          <t>(none — JS-rendered page)</t>
+          <t>[base64] → images/are-all-electric-vehicle-chargers-the-same/content_img_01.png</t>
         </is>
       </c>
     </row>
@@ -712,7 +712,7 @@
       </c>
       <c r="L4" s="2" t="inlineStr">
         <is>
-          <t>(none — JS-rendered page)</t>
+          <t>[base64] → images/business-electric-car-charger-guide/content_img_01.png</t>
         </is>
       </c>
     </row>
@@ -744,7 +744,7 @@
       </c>
       <c r="F5" s="3" t="inlineStr">
         <is>
-          <t>https://www.grasen.com/news/ev-charging-monetization</t>
+          <t>https://www.grasen.com/news/ev-charging-monetization-commercial-revenue</t>
         </is>
       </c>
       <c r="G5" s="3" t="inlineStr">
@@ -774,7 +774,7 @@
       </c>
       <c r="L5" s="3" t="inlineStr">
         <is>
-          <t>(none — JS-rendered page)</t>
+          <t>(text only — no embedded images)</t>
         </is>
       </c>
     </row>
@@ -806,7 +806,7 @@
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>https://www.grasen.com/news/top-10-dc-fast-charger-manufacturers-china</t>
+          <t>https://www.grasen.com/news/top-dc-fast-charger-manufacturers-china-2026</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr">
@@ -836,7 +836,7 @@
       </c>
       <c r="L6" s="2" t="inlineStr">
         <is>
-          <t>(none — JS-rendered page)</t>
+          <t>[base64] → images/top-10-dc-fast-charger-manufacturers-china/content_img_01.png</t>
         </is>
       </c>
     </row>
@@ -868,7 +868,7 @@
       </c>
       <c r="F7" s="3" t="inlineStr">
         <is>
-          <t>https://www.grasen.com/news/how-to-use-grasen-app</t>
+          <t>https://www.grasen.com/news/how-to-use-grasen-app-ev-charging-management-for-payment</t>
         </is>
       </c>
       <c r="G7" s="3" t="inlineStr">
@@ -898,7 +898,15 @@
       </c>
       <c r="L7" s="3" t="inlineStr">
         <is>
-          <t>(none — JS-rendered page)</t>
+          <t>[base64] → images/how-to-use-grasen-app/content_img_01.png
+[base64] → images/how-to-use-grasen-app/content_img_02.png
+[base64] → images/how-to-use-grasen-app/content_img_03.png
+[base64] → images/how-to-use-grasen-app/content_img_04.png
+[base64] → images/how-to-use-grasen-app/content_img_05.png
+[base64] → images/how-to-use-grasen-app/content_img_06.png
+[base64] → images/how-to-use-grasen-app/content_img_07.png
+[base64] → images/how-to-use-grasen-app/content_img_08.png
+[base64] → images/how-to-use-grasen-app/content_img_09.png</t>
         </is>
       </c>
     </row>
@@ -930,7 +938,7 @@
       </c>
       <c r="F8" s="2" t="inlineStr">
         <is>
-          <t>https://www.grasen.com/news/grasen-t480q-480kw-4-gun-dc-ev-fast-charger</t>
+          <t>https://www.grasen.com/news/t480q-480kw-4-gun-dc-fast-charger</t>
         </is>
       </c>
       <c r="G8" s="2" t="inlineStr">
@@ -960,7 +968,7 @@
       </c>
       <c r="L8" s="2" t="inlineStr">
         <is>
-          <t>(none — JS-rendered page)</t>
+          <t>(text only — no embedded images)</t>
         </is>
       </c>
     </row>
@@ -992,7 +1000,7 @@
       </c>
       <c r="F9" s="3" t="inlineStr">
         <is>
-          <t>https://www.grasen.com/news/dual-gun-dc-fast-charger-power-sharing</t>
+          <t>https://www.grasen.com/news/dual-gun-dc-fast-charger-power-sharing-grasen</t>
         </is>
       </c>
       <c r="G9" s="3" t="inlineStr">
@@ -1022,7 +1030,7 @@
       </c>
       <c r="L9" s="3" t="inlineStr">
         <is>
-          <t>(none — JS-rendered page)</t>
+          <t>(text only — no embedded images)</t>
         </is>
       </c>
     </row>
@@ -1054,7 +1062,7 @@
       </c>
       <c r="F10" s="2" t="inlineStr">
         <is>
-          <t>https://www.grasen.com/news/ccs2-dc-fast-chargers-commercial-stations</t>
+          <t>https://www.grasen.com/news/ccs2-dc-fast-charger-commercial-ev-charging</t>
         </is>
       </c>
       <c r="G10" s="2" t="inlineStr">
@@ -1084,7 +1092,7 @@
       </c>
       <c r="L10" s="2" t="inlineStr">
         <is>
-          <t>(none — JS-rendered page)</t>
+          <t>(text only — no embedded images)</t>
         </is>
       </c>
     </row>
@@ -1116,7 +1124,7 @@
       </c>
       <c r="F11" s="3" t="inlineStr">
         <is>
-          <t>https://www.grasen.com/news/grasen-canton-fair-140th-2026</t>
+          <t>https://www.grasen.com/news/grasen-140th-canton-fair-2026</t>
         </is>
       </c>
       <c r="G11" s="3" t="inlineStr">
@@ -1146,7 +1154,7 @@
       </c>
       <c r="L11" s="3" t="inlineStr">
         <is>
-          <t>(none — JS-rendered page)</t>
+          <t>(text only — no embedded images)</t>
         </is>
       </c>
     </row>

</xml_diff>